<commit_message>
Update question bank via TIMSS admin
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1217,9 +1217,44 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>text-choice</v>
+      </c>
+      <c r="C24" t="str">
+        <v>測試</v>
+      </c>
+      <c r="D24" t="str">
+        <v>測試</v>
+      </c>
+      <c r="E24" t="str">
+        <v>減少營養流失</v>
+      </c>
+      <c r="F24" t="str">
+        <v>增加吸引空氣中水分的機會</v>
+      </c>
+      <c r="G24" t="str">
+        <v>減少水分流失</v>
+      </c>
+      <c r="H24" t="str">
+        <v>怕太陽曬</v>
+      </c>
+      <c r="I24" t="str">
+        <v>C</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>